<commit_message>
save files with fossil and power demand
</commit_message>
<xml_diff>
--- a/Scripts/Industry/Results_per_Country/2030_AT.xlsx
+++ b/Scripts/Industry/Results_per_Country/2030_AT.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,85 +452,117 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1465.462811187185</v>
+        <v>17091.40720524144</v>
       </c>
       <c r="C2" t="n">
-        <v>2458.815200492646</v>
+        <v>8273.120404398047</v>
       </c>
       <c r="D2" t="n">
-        <v>3973.532412259082</v>
+        <v>9560.575638196082</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1465.462811187185</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+        <v>2436.779093369591</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5814.3052039054</v>
+      </c>
+      <c r="D3" t="n">
+        <v>739.4622629804579</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Methanol</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="n">
-        <v>33.93168714694505</v>
-      </c>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1465.462811187185</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Methanol</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>2424.883513345701</v>
+        <v>33.93168714694505</v>
       </c>
       <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Biomass</t>
+          <t>Ammonia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
-        <v>3434.912305263911</v>
-      </c>
+      <c r="C6" t="n">
+        <v>2424.883513345701</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Biogas</t>
+          <t>Biomass</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>411.770166210904</v>
+        <v>3434.912305263911</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Biogas</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
+        <v>411.770166210904</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
         <v>126.8499407842673</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Fossil Rest</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>13189.16530068466</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4847.580962956541</v>
       </c>
     </row>
   </sheetData>

</xml_diff>